<commit_message>
phase 3-5 of clustering done, plus stamp added
</commit_message>
<xml_diff>
--- a/Coordinates for map.xlsx
+++ b/Coordinates for map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentshu-my.sharepoint.com/personal/handliem_shu_edu/Documents/Documents/Codes/Project1v1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="8_{C0B26E65-74C6-4646-9754-ED42DD1EC572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{941493C2-E7DA-4091-AB38-BE4A9212AAB5}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{C0B26E65-74C6-4646-9754-ED42DD1EC572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{500710E1-4A70-4A55-B9A1-EED41800D27F}"/>
   <bookViews>
-    <workbookView xWindow="470" yWindow="200" windowWidth="18740" windowHeight="11280" xr2:uid="{60A329A8-B80B-4660-B992-29E8C93735F0}"/>
+    <workbookView xWindow="230" yWindow="720" windowWidth="18970" windowHeight="11280" xr2:uid="{60A329A8-B80B-4660-B992-29E8C93735F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Name</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>Nowhere</t>
+  </si>
+  <si>
+    <t>Test2</t>
+  </si>
+  <si>
+    <t>Somewhere near NY</t>
   </si>
 </sst>
 </file>
@@ -112,6 +118,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -431,7 +441,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2562405C-7E72-4486-BA67-46A6B97B33A8}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.1796875" customWidth="1"/>
@@ -483,6 +493,20 @@
         <v>7</v>
       </c>
     </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>4900</v>
+      </c>
+      <c r="C4">
+        <v>5100</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add caching for zoom
</commit_message>
<xml_diff>
--- a/Coordinates for map.xlsx
+++ b/Coordinates for map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentshu-my.sharepoint.com/personal/handliem_shu_edu/Documents/Documents/Codes/Project1v1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{C0B26E65-74C6-4646-9754-ED42DD1EC572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{500710E1-4A70-4A55-B9A1-EED41800D27F}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="8_{C0B26E65-74C6-4646-9754-ED42DD1EC572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5ECCE00B-9EEA-4FA8-8B1B-8063F16BA63A}"/>
   <bookViews>
     <workbookView xWindow="230" yWindow="720" windowWidth="18970" windowHeight="11280" xr2:uid="{60A329A8-B80B-4660-B992-29E8C93735F0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Name</t>
   </si>
@@ -66,6 +66,12 @@
   </si>
   <si>
     <t>Somewhere near NY</t>
+  </si>
+  <si>
+    <t>Coordinate X halfsize</t>
+  </si>
+  <si>
+    <t>Coordinate Y halfsize</t>
   </si>
 </sst>
 </file>
@@ -118,10 +124,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -441,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2562405C-7E72-4486-BA67-46A6B97B33A8}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.1796875" customWidth="1"/>
@@ -449,9 +451,10 @@
     <col min="3" max="3" width="17" customWidth="1"/>
     <col min="4" max="4" width="17.36328125" customWidth="1"/>
     <col min="5" max="5" width="17.453125" customWidth="1"/>
+    <col min="6" max="6" width="17.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -464,8 +467,14 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -478,8 +487,16 @@
       <c r="D2" t="s">
         <v>5</v>
       </c>
+      <c r="E2">
+        <f>ROUND(B2/2,0)</f>
+        <v>2460</v>
+      </c>
+      <c r="F2">
+        <f t="shared" ref="F2:F4" si="0">ROUND(C2/2,0)</f>
+        <v>2577</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -492,8 +509,16 @@
       <c r="D3" t="s">
         <v>7</v>
       </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E4" si="1">ROUND(B3/2,0)</f>
+        <v>4500</v>
+      </c>
+      <c r="F3">
+        <f t="shared" si="0"/>
+        <v>1750</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -505,6 +530,14 @@
       </c>
       <c r="D4" t="s">
         <v>9</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="1"/>
+        <v>2450</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>2550</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added map markers for all people/objects
</commit_message>
<xml_diff>
--- a/Coordinates for map.xlsx
+++ b/Coordinates for map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentshu-my.sharepoint.com/personal/handliem_shu_edu/Documents/Documents/Codes/Project1v1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{C0B26E65-74C6-4646-9754-ED42DD1EC572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5ECCE00B-9EEA-4FA8-8B1B-8063F16BA63A}"/>
+  <xr:revisionPtr revIDLastSave="127" documentId="8_{C0B26E65-74C6-4646-9754-ED42DD1EC572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18606B94-8D61-44CF-B23B-3FC67BD21982}"/>
   <bookViews>
-    <workbookView xWindow="230" yWindow="720" windowWidth="18970" windowHeight="11280" xr2:uid="{60A329A8-B80B-4660-B992-29E8C93735F0}"/>
+    <workbookView xWindow="230" yWindow="380" windowWidth="18970" windowHeight="11280" xr2:uid="{60A329A8-B80B-4660-B992-29E8C93735F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Name</t>
   </si>
@@ -72,19 +72,130 @@
   </si>
   <si>
     <t>Coordinate Y halfsize</t>
+  </si>
+  <si>
+    <t>Chen Dingshan</t>
+  </si>
+  <si>
+    <t>Chow Studio</t>
+  </si>
+  <si>
+    <t>Dr. Henry Rosin</t>
+  </si>
+  <si>
+    <t>Dr. Jerry Silver</t>
+  </si>
+  <si>
+    <t>Dr. John Tcheng</t>
+  </si>
+  <si>
+    <t>Dr. Leon Chang</t>
+  </si>
+  <si>
+    <t>Dr. Marvin Boris</t>
+  </si>
+  <si>
+    <t>Dr. Paul Singer</t>
+  </si>
+  <si>
+    <t>James Stein</t>
+  </si>
+  <si>
+    <t>Jung Ying Tsao</t>
+  </si>
+  <si>
+    <t>Liu Yen-T'ao</t>
+  </si>
+  <si>
+    <t>Anonymous</t>
+  </si>
+  <si>
+    <t>Ch'eng Chieh-tzu</t>
+  </si>
+  <si>
+    <t>Chang Dai-chien</t>
+  </si>
+  <si>
+    <t>Mr. and Mrs. C.C. Wang</t>
+  </si>
+  <si>
+    <t>Mr. and Mrs. Lin Hsun</t>
+  </si>
+  <si>
+    <t>Mr. and Mrs. Zen Zuh Li</t>
+  </si>
+  <si>
+    <t>Mr. David Kwo</t>
+  </si>
+  <si>
+    <t>Mr. I-Chao Chu</t>
+  </si>
+  <si>
+    <t>Mr. Johnson S.S Chow</t>
+  </si>
+  <si>
+    <t>Mrs. Frank L. Babbott</t>
+  </si>
+  <si>
+    <t>Mrs. Matthew A. Smith</t>
+  </si>
+  <si>
+    <t>Mrs. S.I. Hsiung</t>
+  </si>
+  <si>
+    <t>Peter and Mary White</t>
+  </si>
+  <si>
+    <t>Prof. Chan Ku-Nien</t>
+  </si>
+  <si>
+    <t>Prof. Chao Shao-an</t>
+  </si>
+  <si>
+    <t>Prof. Charles Chu</t>
+  </si>
+  <si>
+    <t>Prof. I-Pong Van</t>
+  </si>
+  <si>
+    <t>Prof. Wang Fangyu</t>
+  </si>
+  <si>
+    <t>Rev. Peter P.S. Ching</t>
+  </si>
+  <si>
+    <t>Robert Sistrunk</t>
+  </si>
+  <si>
+    <t>Rose Woo Hui Ching</t>
+  </si>
+  <si>
+    <t>Wang Chuang-wei</t>
+  </si>
+  <si>
+    <t>George Young</t>
+  </si>
+  <si>
+    <t>Morton Gordon</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -107,8 +218,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -443,10 +557,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2562405C-7E72-4486-BA67-46A6B97B33A8}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.1796875" customWidth="1"/>
+    <col min="1" max="1" width="29.453125" customWidth="1"/>
     <col min="2" max="2" width="17.54296875" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
     <col min="4" max="4" width="17.36328125" customWidth="1"/>
@@ -540,7 +654,389 @@
         <v>2550</v>
       </c>
     </row>
+    <row r="6" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>6378</v>
+      </c>
+      <c r="F7">
+        <v>2933</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8">
+        <v>6366</v>
+      </c>
+      <c r="F8">
+        <v>2937</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9">
+        <v>6378</v>
+      </c>
+      <c r="F9">
+        <v>2939</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10">
+        <v>2334</v>
+      </c>
+      <c r="F10">
+        <v>2930</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11">
+        <v>2453</v>
+      </c>
+      <c r="F11">
+        <v>2573</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12">
+        <v>2454</v>
+      </c>
+      <c r="F12">
+        <v>2571</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13">
+        <v>2251</v>
+      </c>
+      <c r="F13">
+        <v>2616</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14">
+        <v>2467</v>
+      </c>
+      <c r="F14">
+        <v>2575</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15">
+        <v>2469</v>
+      </c>
+      <c r="F15">
+        <v>2572</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16">
+        <v>2451</v>
+      </c>
+      <c r="F16">
+        <v>2576</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17">
+        <v>2466</v>
+      </c>
+      <c r="F17">
+        <v>2573</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E18">
+        <v>2461</v>
+      </c>
+      <c r="F18">
+        <v>2573</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E19">
+        <v>1495</v>
+      </c>
+      <c r="F19">
+        <v>2648</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20">
+        <v>6377</v>
+      </c>
+      <c r="F20">
+        <v>2928</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E21">
+        <v>2449</v>
+      </c>
+      <c r="F21">
+        <v>2575</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22">
+        <v>2463</v>
+      </c>
+      <c r="F22">
+        <v>2575</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23">
+        <v>2468</v>
+      </c>
+      <c r="F23">
+        <v>2574</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24">
+        <v>2461</v>
+      </c>
+      <c r="F24">
+        <v>2577</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E25">
+        <v>2454</v>
+      </c>
+      <c r="F25">
+        <v>2571</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E26">
+        <v>2451</v>
+      </c>
+      <c r="F26">
+        <v>2573</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E27">
+        <v>1566</v>
+      </c>
+      <c r="F27">
+        <v>2744</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E28">
+        <v>2450</v>
+      </c>
+      <c r="F28">
+        <v>2574</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E29">
+        <v>2429</v>
+      </c>
+      <c r="F29">
+        <v>2569</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E30">
+        <v>1486</v>
+      </c>
+      <c r="F30">
+        <v>2653</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E31">
+        <v>3941</v>
+      </c>
+      <c r="F31">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32">
+        <v>2259</v>
+      </c>
+      <c r="F32">
+        <v>2508</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E33">
+        <v>6229</v>
+      </c>
+      <c r="F33">
+        <v>2993</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E34">
+        <v>2488</v>
+      </c>
+      <c r="F34">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E35">
+        <v>6228</v>
+      </c>
+      <c r="F35">
+        <v>2989</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E36">
+        <v>2449</v>
+      </c>
+      <c r="F36">
+        <v>2573</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E37">
+        <v>2467</v>
+      </c>
+      <c r="F37">
+        <v>2572</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E38">
+        <v>2460</v>
+      </c>
+      <c r="F38">
+        <v>2574</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A39" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E39">
+        <v>6228</v>
+      </c>
+      <c r="F39">
+        <v>2984</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A40" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E40">
+        <v>6380</v>
+      </c>
+      <c r="F40">
+        <v>2930</v>
+      </c>
+    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:A40">
+    <sortCondition ref="A6:A40"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restore Excel half-size coordinate columns
</commit_message>
<xml_diff>
--- a/Coordinates for map.xlsx
+++ b/Coordinates for map.xlsx
@@ -14,10 +14,7 @@
   <fonts count="1">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="1">
@@ -69,40 +66,50 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Coordinate X halfsize</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Coordinate Y halfsize</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Image 1 filename</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Image 2 filename</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Image 3 filename</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Image 4 filename</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Image 5 filename</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Image 6 filename</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Image 7 filename</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Image 8 filename</t>
         </is>
@@ -115,41 +122,37 @@
         </is>
       </c>
       <c r="B2">
-        <v>4920.0</v>
+        <v>4920</v>
       </c>
       <c r="C2">
-        <v>5153.0</v>
+        <v>5153</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2">
+        <v>2460</v>
+      </c>
+      <c r="F2">
+        <v>2576</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>1-letter-product-pic.jpg</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2-v4-460px-Write-a-Friendly-Letter-Step-4-Version-6 - Copy.jpg</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>3-v4-460px-Write-a-Friendly-Letter-Step-4-Version-6.jpg</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t/>
@@ -161,6 +164,16 @@
         </is>
       </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -173,52 +186,58 @@
         </is>
       </c>
       <c r="B3">
-        <v>9000.0</v>
+        <v>9000</v>
       </c>
       <c r="C3">
-        <v>3500.0</v>
+        <v>3500</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>Nowhere</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3">
+        <v>4500</v>
+      </c>
+      <c r="F3">
+        <v>1750</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>1-77.10.21 Photograph Obverse.jpg</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>2-stamp_demo.png</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>3-letter-product-pic.jpg</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>4-stamp_demo - Copy (4).png</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>5-stamp_demo - Copy (2).png</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>6-77.10.21_artist_letter.png</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>7-stamp_demo - Copy (3).png</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>8-letter-product-pic - Copy.jpg</t>
         </is>
@@ -231,31 +250,27 @@
         </is>
       </c>
       <c r="B4">
-        <v>4900.0</v>
+        <v>4900</v>
       </c>
       <c r="C4">
-        <v>5100.0</v>
+        <v>5100</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>Somewhere near NY</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4">
+        <v>2450</v>
+      </c>
+      <c r="F4">
+        <v>2550</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>1-letter-product-pic.jpg</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t/>
@@ -277,6 +292,16 @@
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -289,25 +314,21 @@
         </is>
       </c>
       <c r="B5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -335,6 +356,16 @@
         </is>
       </c>
       <c r="L5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -347,25 +378,21 @@
         </is>
       </c>
       <c r="B6">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C6">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -393,6 +420,16 @@
         </is>
       </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -405,25 +442,21 @@
         </is>
       </c>
       <c r="B7">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C7">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -451,6 +484,16 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -463,25 +506,21 @@
         </is>
       </c>
       <c r="B8">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C8">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -509,6 +548,16 @@
         </is>
       </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -521,25 +570,21 @@
         </is>
       </c>
       <c r="B9">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C9">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -567,6 +612,16 @@
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -579,25 +634,21 @@
         </is>
       </c>
       <c r="B10">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C10">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -625,6 +676,16 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -637,25 +698,21 @@
         </is>
       </c>
       <c r="B11">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C11">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -683,6 +740,16 @@
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -695,25 +762,21 @@
         </is>
       </c>
       <c r="B12">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C12">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -741,6 +804,16 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -753,25 +826,21 @@
         </is>
       </c>
       <c r="B13">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C13">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -799,6 +868,16 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -811,25 +890,21 @@
         </is>
       </c>
       <c r="B14">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C14">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -857,6 +932,16 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -869,25 +954,21 @@
         </is>
       </c>
       <c r="B15">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C15">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -915,6 +996,16 @@
         </is>
       </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -927,25 +1018,21 @@
         </is>
       </c>
       <c r="B16">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C16">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -973,6 +1060,16 @@
         </is>
       </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -985,25 +1082,21 @@
         </is>
       </c>
       <c r="B17">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C17">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1031,6 +1124,16 @@
         </is>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1043,25 +1146,21 @@
         </is>
       </c>
       <c r="B18">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C18">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1089,6 +1188,16 @@
         </is>
       </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1101,25 +1210,21 @@
         </is>
       </c>
       <c r="B19">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C19">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1147,6 +1252,16 @@
         </is>
       </c>
       <c r="L19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1159,25 +1274,21 @@
         </is>
       </c>
       <c r="B20">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C20">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1205,6 +1316,16 @@
         </is>
       </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1217,25 +1338,21 @@
         </is>
       </c>
       <c r="B21">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C21">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1263,6 +1380,16 @@
         </is>
       </c>
       <c r="L21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1275,25 +1402,21 @@
         </is>
       </c>
       <c r="B22">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C22">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1321,6 +1444,16 @@
         </is>
       </c>
       <c r="L22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1333,25 +1466,21 @@
         </is>
       </c>
       <c r="B23">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C23">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1379,6 +1508,16 @@
         </is>
       </c>
       <c r="L23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1391,25 +1530,21 @@
         </is>
       </c>
       <c r="B24">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C24">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1437,6 +1572,16 @@
         </is>
       </c>
       <c r="L24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1449,25 +1594,21 @@
         </is>
       </c>
       <c r="B25">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C25">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1495,6 +1636,16 @@
         </is>
       </c>
       <c r="L25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1507,25 +1658,21 @@
         </is>
       </c>
       <c r="B26">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C26">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1553,6 +1700,16 @@
         </is>
       </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1565,25 +1722,21 @@
         </is>
       </c>
       <c r="B27">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C27">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1611,6 +1764,16 @@
         </is>
       </c>
       <c r="L27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1623,25 +1786,21 @@
         </is>
       </c>
       <c r="B28">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C28">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1669,6 +1828,16 @@
         </is>
       </c>
       <c r="L28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1681,25 +1850,21 @@
         </is>
       </c>
       <c r="B29">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C29">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1727,6 +1892,16 @@
         </is>
       </c>
       <c r="L29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1739,25 +1914,21 @@
         </is>
       </c>
       <c r="B30">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C30">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1785,6 +1956,16 @@
         </is>
       </c>
       <c r="L30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1797,25 +1978,21 @@
         </is>
       </c>
       <c r="B31">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C31">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1843,6 +2020,16 @@
         </is>
       </c>
       <c r="L31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1855,25 +2042,21 @@
         </is>
       </c>
       <c r="B32">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C32">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1901,6 +2084,16 @@
         </is>
       </c>
       <c r="L32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1913,25 +2106,21 @@
         </is>
       </c>
       <c r="B33">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C33">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E33">
+        <v>0</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1959,6 +2148,16 @@
         </is>
       </c>
       <c r="L33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1971,25 +2170,21 @@
         </is>
       </c>
       <c r="B34">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C34">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -2017,6 +2212,16 @@
         </is>
       </c>
       <c r="L34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2029,25 +2234,21 @@
         </is>
       </c>
       <c r="B35">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C35">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2075,6 +2276,16 @@
         </is>
       </c>
       <c r="L35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2087,25 +2298,21 @@
         </is>
       </c>
       <c r="B36">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C36">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2133,6 +2340,16 @@
         </is>
       </c>
       <c r="L36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2145,25 +2362,21 @@
         </is>
       </c>
       <c r="B37">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C37">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2191,6 +2404,16 @@
         </is>
       </c>
       <c r="L37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2203,25 +2426,21 @@
         </is>
       </c>
       <c r="B38">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C38">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2249,6 +2468,16 @@
         </is>
       </c>
       <c r="L38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2261,41 +2490,37 @@
         </is>
       </c>
       <c r="B39">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C39">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39">
+        <v>0</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39" t="inlineStr">
         <is>
           <t>1-77.10.16 Photograph Obverse.png</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>2-77.10.2_letter2_2.png</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>3-77.10.2_letter page 2.png</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="J39" t="inlineStr">
         <is>
           <t/>
@@ -2307,6 +2532,16 @@
         </is>
       </c>
       <c r="L39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
Restore workbook coordinate values
</commit_message>
<xml_diff>
--- a/Coordinates for map.xlsx
+++ b/Coordinates for map.xlsx
@@ -136,7 +136,7 @@
         <v>2460</v>
       </c>
       <c r="F2">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -378,10 +378,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>12756</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>5866</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -389,10 +389,10 @@
         </is>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>6378</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>2933</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -442,10 +442,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>12732</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>5874</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -453,10 +453,10 @@
         </is>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>6366</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>2937</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -506,10 +506,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>12756</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>5878</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>6378</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>2939</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -570,10 +570,10 @@
         </is>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>4668</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>5860</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -581,10 +581,10 @@
         </is>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>2334</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>2930</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -634,10 +634,10 @@
         </is>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>4906</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>5146</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -645,10 +645,10 @@
         </is>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>2453</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>2573</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -698,10 +698,10 @@
         </is>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>4908</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>5142</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -709,10 +709,10 @@
         </is>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>2454</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>2571</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -762,10 +762,10 @@
         </is>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>4502</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>5232</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -773,10 +773,10 @@
         </is>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>2251</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>2616</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -826,10 +826,10 @@
         </is>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>4934</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>5150</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -837,10 +837,10 @@
         </is>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>2467</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>2575</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -890,10 +890,10 @@
         </is>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>4938</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>5144</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -901,10 +901,10 @@
         </is>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>2469</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>2572</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -954,10 +954,10 @@
         </is>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>4902</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>5152</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -965,10 +965,10 @@
         </is>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>2451</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>2576</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1018,10 +1018,10 @@
         </is>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>4932</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>5146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         </is>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>2466</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>2573</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         </is>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>4922</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>5146</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>2461</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>2573</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1146,10 +1146,10 @@
         </is>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>2990</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>5296</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1157,10 +1157,10 @@
         </is>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>1495</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>2648</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1210,10 +1210,10 @@
         </is>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>12754</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>5856</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1221,10 +1221,10 @@
         </is>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>6377</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>2928</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1274,10 +1274,10 @@
         </is>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>4898</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>5150</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1285,10 +1285,10 @@
         </is>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>2449</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>2575</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1338,10 +1338,10 @@
         </is>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>4926</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>5150</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1349,10 +1349,10 @@
         </is>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>2463</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>2575</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1402,10 +1402,10 @@
         </is>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>4936</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>5148</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1413,10 +1413,10 @@
         </is>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>2468</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>2574</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1466,10 +1466,10 @@
         </is>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>4922</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>5154</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1477,10 +1477,10 @@
         </is>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>2461</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>2577</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1530,10 +1530,10 @@
         </is>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>4908</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>5142</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1541,10 +1541,10 @@
         </is>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>2454</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>2571</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1594,10 +1594,10 @@
         </is>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>4902</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>5146</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1605,10 +1605,10 @@
         </is>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>2451</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>2573</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1658,10 +1658,10 @@
         </is>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>3132</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>5488</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1669,10 +1669,10 @@
         </is>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>1566</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>2744</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1722,10 +1722,10 @@
         </is>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>4900</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>5148</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1733,10 +1733,10 @@
         </is>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>2450</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>2574</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1786,10 +1786,10 @@
         </is>
       </c>
       <c r="B28">
-        <v>0</v>
+        <v>4858</v>
       </c>
       <c r="C28">
-        <v>0</v>
+        <v>5138</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1797,10 +1797,10 @@
         </is>
       </c>
       <c r="E28">
-        <v>0</v>
+        <v>2429</v>
       </c>
       <c r="F28">
-        <v>0</v>
+        <v>2569</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1850,10 +1850,10 @@
         </is>
       </c>
       <c r="B29">
-        <v>0</v>
+        <v>2972</v>
       </c>
       <c r="C29">
-        <v>0</v>
+        <v>5306</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1861,10 +1861,10 @@
         </is>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>1486</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>2653</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1914,10 +1914,10 @@
         </is>
       </c>
       <c r="B30">
-        <v>0</v>
+        <v>7882</v>
       </c>
       <c r="C30">
-        <v>0</v>
+        <v>4500</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1925,10 +1925,10 @@
         </is>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>3941</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>2250</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1978,10 +1978,10 @@
         </is>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>4518</v>
       </c>
       <c r="C31">
-        <v>0</v>
+        <v>5016</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1989,10 +1989,10 @@
         </is>
       </c>
       <c r="E31">
-        <v>0</v>
+        <v>2259</v>
       </c>
       <c r="F31">
-        <v>0</v>
+        <v>2508</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -2042,10 +2042,10 @@
         </is>
       </c>
       <c r="B32">
-        <v>0</v>
+        <v>12458</v>
       </c>
       <c r="C32">
-        <v>0</v>
+        <v>5986</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2053,10 +2053,10 @@
         </is>
       </c>
       <c r="E32">
-        <v>0</v>
+        <v>6229</v>
       </c>
       <c r="F32">
-        <v>0</v>
+        <v>2993</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -2106,10 +2106,10 @@
         </is>
       </c>
       <c r="B33">
-        <v>0</v>
+        <v>4976</v>
       </c>
       <c r="C33">
-        <v>0</v>
+        <v>5112</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2117,10 +2117,10 @@
         </is>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>2488</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>2556</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -2170,10 +2170,10 @@
         </is>
       </c>
       <c r="B34">
-        <v>0</v>
+        <v>12456</v>
       </c>
       <c r="C34">
-        <v>0</v>
+        <v>5978</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2181,10 +2181,10 @@
         </is>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>6228</v>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>2989</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -2234,10 +2234,10 @@
         </is>
       </c>
       <c r="B35">
-        <v>0</v>
+        <v>4898</v>
       </c>
       <c r="C35">
-        <v>0</v>
+        <v>5146</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2245,10 +2245,10 @@
         </is>
       </c>
       <c r="E35">
-        <v>0</v>
+        <v>2449</v>
       </c>
       <c r="F35">
-        <v>0</v>
+        <v>2573</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2298,10 +2298,10 @@
         </is>
       </c>
       <c r="B36">
-        <v>0</v>
+        <v>4934</v>
       </c>
       <c r="C36">
-        <v>0</v>
+        <v>5144</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2309,10 +2309,10 @@
         </is>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>2467</v>
       </c>
       <c r="F36">
-        <v>0</v>
+        <v>2572</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2362,10 +2362,10 @@
         </is>
       </c>
       <c r="B37">
-        <v>0</v>
+        <v>4920</v>
       </c>
       <c r="C37">
-        <v>0</v>
+        <v>5148</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2373,10 +2373,10 @@
         </is>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>2460</v>
       </c>
       <c r="F37">
-        <v>0</v>
+        <v>2574</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2426,10 +2426,10 @@
         </is>
       </c>
       <c r="B38">
-        <v>0</v>
+        <v>12456</v>
       </c>
       <c r="C38">
-        <v>0</v>
+        <v>5968</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2437,10 +2437,10 @@
         </is>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>6228</v>
       </c>
       <c r="F38">
-        <v>0</v>
+        <v>2984</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2490,10 +2490,10 @@
         </is>
       </c>
       <c r="B39">
-        <v>0</v>
+        <v>12760</v>
       </c>
       <c r="C39">
-        <v>0</v>
+        <v>5860</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2501,10 +2501,10 @@
         </is>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>6380</v>
       </c>
       <c r="F39">
-        <v>0</v>
+        <v>2930</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>

</xml_diff>